<commit_message>
Append new results, 1 spreadsheet for all events, medals and WR
</commit_message>
<xml_diff>
--- a/pages/video_analysis/IP_Master_Men.xlsx
+++ b/pages/video_analysis/IP_Master_Men.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sportnzgroup-my.sharepoint.com/personal/anja_kuys_hpsnz_org_nz/Documents/Desktop/Scripts/CNZPD/pages/video_analysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="11_F1FC6792D89E629903ED24B2C9460C765188C8B3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D2D1CB14-47C1-4953-96E7-B64BD2730C23}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="11_F1FC6792D89E629903ED24B2C9460C765188C8B3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2FD742A7-85B4-4B4C-A004-06A21C31CBA8}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="1620" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="778" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="781" uniqueCount="20">
   <si>
     <t>Title</t>
   </si>
@@ -71,6 +71,15 @@
   </si>
   <si>
     <t>26-07-31 Glasgow CWG Morton Q</t>
+  </si>
+  <si>
+    <t>https://youtu.be/qCTIxXtG0Lg</t>
+  </si>
+  <si>
+    <t>https://youtu.be/yjVZcfO11qw</t>
+  </si>
+  <si>
+    <t>https://youtu.be/z7zcj4I4qic</t>
   </si>
 </sst>
 </file>
@@ -413,12 +422,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I321"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="32.58203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -444,7 +453,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -470,7 +479,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -493,7 +502,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -516,7 +525,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -539,7 +548,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -562,7 +571,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -585,7 +594,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -608,7 +617,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -631,7 +640,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -654,7 +663,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>8</v>
       </c>
@@ -677,7 +686,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>8</v>
       </c>
@@ -700,7 +709,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>8</v>
       </c>
@@ -723,7 +732,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>8</v>
       </c>
@@ -746,7 +755,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>8</v>
       </c>
@@ -769,7 +778,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>8</v>
       </c>
@@ -792,7 +801,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>8</v>
       </c>
@@ -815,7 +824,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>8</v>
       </c>
@@ -838,7 +847,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>8</v>
       </c>
@@ -861,7 +870,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>8</v>
       </c>
@@ -884,7 +893,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>8</v>
       </c>
@@ -907,7 +916,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>8</v>
       </c>
@@ -930,7 +939,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="23" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>8</v>
       </c>
@@ -953,7 +962,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>8</v>
       </c>
@@ -976,7 +985,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="25" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>8</v>
       </c>
@@ -999,7 +1008,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>8</v>
       </c>
@@ -1022,7 +1031,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="27" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>8</v>
       </c>
@@ -1045,7 +1054,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="28" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>8</v>
       </c>
@@ -1068,7 +1077,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="29" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>8</v>
       </c>
@@ -1091,7 +1100,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="30" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>8</v>
       </c>
@@ -1114,7 +1123,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="31" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>8</v>
       </c>
@@ -1137,7 +1146,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="32" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>8</v>
       </c>
@@ -1160,7 +1169,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="33" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>8</v>
       </c>
@@ -1183,7 +1192,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="34" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>8</v>
       </c>
@@ -1206,7 +1215,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="35" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>8</v>
       </c>
@@ -1229,7 +1238,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="36" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>8</v>
       </c>
@@ -1252,7 +1261,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="37" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>8</v>
       </c>
@@ -1275,7 +1284,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="38" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>8</v>
       </c>
@@ -1298,7 +1307,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="39" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>8</v>
       </c>
@@ -1321,7 +1330,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="40" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>8</v>
       </c>
@@ -1344,7 +1353,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="41" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>8</v>
       </c>
@@ -1367,7 +1376,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="42" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>8</v>
       </c>
@@ -1390,7 +1399,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="43" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>8</v>
       </c>
@@ -1413,7 +1422,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="44" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>8</v>
       </c>
@@ -1436,7 +1445,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="45" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>8</v>
       </c>
@@ -1459,7 +1468,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="46" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>8</v>
       </c>
@@ -1482,7 +1491,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="47" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>8</v>
       </c>
@@ -1505,7 +1514,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="48" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>8</v>
       </c>
@@ -1528,7 +1537,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="49" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>8</v>
       </c>
@@ -1551,7 +1560,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="50" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>8</v>
       </c>
@@ -1574,7 +1583,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="51" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>8</v>
       </c>
@@ -1597,7 +1606,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="52" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>8</v>
       </c>
@@ -1620,7 +1629,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="53" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>8</v>
       </c>
@@ -1643,7 +1652,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="54" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>8</v>
       </c>
@@ -1666,7 +1675,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="55" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>8</v>
       </c>
@@ -1689,7 +1698,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="56" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>8</v>
       </c>
@@ -1712,7 +1721,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="57" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>8</v>
       </c>
@@ -1735,7 +1744,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="58" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>8</v>
       </c>
@@ -1758,7 +1767,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="59" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>8</v>
       </c>
@@ -1781,7 +1790,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="60" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>8</v>
       </c>
@@ -1804,7 +1813,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="61" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>8</v>
       </c>
@@ -1827,7 +1836,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="62" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>8</v>
       </c>
@@ -1850,7 +1859,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="63" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>8</v>
       </c>
@@ -1873,7 +1882,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="64" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>8</v>
       </c>
@@ -1896,7 +1905,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="65" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>8</v>
       </c>
@@ -1919,7 +1928,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="66" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>11</v>
       </c>
@@ -1945,7 +1954,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="67" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>11</v>
       </c>
@@ -1968,7 +1977,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="68" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>11</v>
       </c>
@@ -1991,7 +2000,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="69" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>11</v>
       </c>
@@ -2014,7 +2023,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="70" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>11</v>
       </c>
@@ -2037,7 +2046,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="71" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>11</v>
       </c>
@@ -2060,7 +2069,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="72" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>11</v>
       </c>
@@ -2083,7 +2092,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="73" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>11</v>
       </c>
@@ -2106,7 +2115,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="74" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>11</v>
       </c>
@@ -2129,7 +2138,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="75" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>11</v>
       </c>
@@ -2152,7 +2161,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="76" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>11</v>
       </c>
@@ -2175,7 +2184,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="77" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>11</v>
       </c>
@@ -2198,7 +2207,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="78" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>11</v>
       </c>
@@ -2221,7 +2230,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="79" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>11</v>
       </c>
@@ -2244,7 +2253,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="80" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>11</v>
       </c>
@@ -2267,7 +2276,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="81" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>11</v>
       </c>
@@ -2290,7 +2299,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="82" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>11</v>
       </c>
@@ -2313,7 +2322,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="83" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>11</v>
       </c>
@@ -2336,7 +2345,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="84" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>11</v>
       </c>
@@ -2359,7 +2368,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="85" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>11</v>
       </c>
@@ -2382,7 +2391,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="86" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>11</v>
       </c>
@@ -2405,7 +2414,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="87" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>11</v>
       </c>
@@ -2428,7 +2437,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="88" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>11</v>
       </c>
@@ -2451,7 +2460,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="89" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>11</v>
       </c>
@@ -2474,7 +2483,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="90" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>11</v>
       </c>
@@ -2497,7 +2506,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="91" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>11</v>
       </c>
@@ -2520,7 +2529,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="92" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>11</v>
       </c>
@@ -2543,7 +2552,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="93" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>11</v>
       </c>
@@ -2566,7 +2575,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="94" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>11</v>
       </c>
@@ -2589,7 +2598,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="95" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>11</v>
       </c>
@@ -2612,7 +2621,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="96" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>11</v>
       </c>
@@ -2635,7 +2644,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="97" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>11</v>
       </c>
@@ -2658,7 +2667,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="98" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
         <v>11</v>
       </c>
@@ -2681,7 +2690,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="99" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
         <v>11</v>
       </c>
@@ -2704,7 +2713,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="100" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
         <v>11</v>
       </c>
@@ -2727,7 +2736,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="101" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
         <v>11</v>
       </c>
@@ -2750,7 +2759,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="102" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
         <v>11</v>
       </c>
@@ -2773,7 +2782,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="103" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
         <v>11</v>
       </c>
@@ -2796,7 +2805,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="104" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
         <v>11</v>
       </c>
@@ -2819,7 +2828,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="105" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
         <v>11</v>
       </c>
@@ -2842,7 +2851,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="106" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
         <v>11</v>
       </c>
@@ -2865,7 +2874,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="107" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
         <v>11</v>
       </c>
@@ -2888,7 +2897,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="108" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
         <v>11</v>
       </c>
@@ -2911,7 +2920,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="109" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
         <v>11</v>
       </c>
@@ -2934,7 +2943,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="110" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
         <v>11</v>
       </c>
@@ -2957,7 +2966,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="111" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
         <v>11</v>
       </c>
@@ -2980,7 +2989,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="112" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
         <v>11</v>
       </c>
@@ -3003,7 +3012,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="113" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
         <v>11</v>
       </c>
@@ -3026,7 +3035,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="114" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
         <v>11</v>
       </c>
@@ -3049,7 +3058,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="115" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
         <v>11</v>
       </c>
@@ -3072,7 +3081,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="116" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
         <v>11</v>
       </c>
@@ -3095,7 +3104,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="117" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
         <v>11</v>
       </c>
@@ -3118,7 +3127,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="118" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
         <v>11</v>
       </c>
@@ -3141,7 +3150,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="119" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
         <v>11</v>
       </c>
@@ -3164,7 +3173,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="120" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
         <v>11</v>
       </c>
@@ -3187,7 +3196,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="121" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
         <v>11</v>
       </c>
@@ -3210,7 +3219,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="122" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
         <v>11</v>
       </c>
@@ -3233,7 +3242,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="123" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
         <v>11</v>
       </c>
@@ -3256,7 +3265,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="124" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A124" t="s">
         <v>11</v>
       </c>
@@ -3279,7 +3288,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="125" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
         <v>11</v>
       </c>
@@ -3302,7 +3311,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="126" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A126" t="s">
         <v>11</v>
       </c>
@@ -3325,7 +3334,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="127" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A127" t="s">
         <v>11</v>
       </c>
@@ -3348,7 +3357,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="128" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A128" t="s">
         <v>11</v>
       </c>
@@ -3371,7 +3380,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="129" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A129" t="s">
         <v>11</v>
       </c>
@@ -3394,7 +3403,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="130" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A130" t="s">
         <v>13</v>
       </c>
@@ -3413,8 +3422,11 @@
       <c r="G130" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="131" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="H130" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="131" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A131" t="s">
         <v>13</v>
       </c>
@@ -3434,7 +3446,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="132" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A132" t="s">
         <v>13</v>
       </c>
@@ -3454,7 +3466,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="133" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A133" t="s">
         <v>13</v>
       </c>
@@ -3474,7 +3486,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="134" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A134" t="s">
         <v>13</v>
       </c>
@@ -3494,7 +3506,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="135" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A135" t="s">
         <v>13</v>
       </c>
@@ -3514,7 +3526,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="136" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A136" t="s">
         <v>13</v>
       </c>
@@ -3534,7 +3546,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="137" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A137" t="s">
         <v>13</v>
       </c>
@@ -3554,7 +3566,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="138" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A138" t="s">
         <v>13</v>
       </c>
@@ -3574,7 +3586,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="139" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A139" t="s">
         <v>13</v>
       </c>
@@ -3594,7 +3606,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="140" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A140" t="s">
         <v>13</v>
       </c>
@@ -3614,7 +3626,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="141" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A141" t="s">
         <v>13</v>
       </c>
@@ -3634,7 +3646,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="142" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A142" t="s">
         <v>13</v>
       </c>
@@ -3654,7 +3666,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="143" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A143" t="s">
         <v>13</v>
       </c>
@@ -3674,7 +3686,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="144" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A144" t="s">
         <v>13</v>
       </c>
@@ -3694,7 +3706,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="145" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A145" t="s">
         <v>13</v>
       </c>
@@ -3714,7 +3726,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="146" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A146" t="s">
         <v>13</v>
       </c>
@@ -3734,7 +3746,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="147" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A147" t="s">
         <v>13</v>
       </c>
@@ -3754,7 +3766,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="148" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A148" t="s">
         <v>13</v>
       </c>
@@ -3774,7 +3786,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="149" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A149" t="s">
         <v>13</v>
       </c>
@@ -3794,7 +3806,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="150" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A150" t="s">
         <v>13</v>
       </c>
@@ -3814,7 +3826,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="151" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A151" t="s">
         <v>13</v>
       </c>
@@ -3834,7 +3846,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="152" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A152" t="s">
         <v>13</v>
       </c>
@@ -3854,7 +3866,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="153" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A153" t="s">
         <v>13</v>
       </c>
@@ -3874,7 +3886,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="154" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A154" t="s">
         <v>13</v>
       </c>
@@ -3894,7 +3906,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="155" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A155" t="s">
         <v>13</v>
       </c>
@@ -3914,7 +3926,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="156" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A156" t="s">
         <v>13</v>
       </c>
@@ -3934,7 +3946,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="157" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A157" t="s">
         <v>13</v>
       </c>
@@ -3954,7 +3966,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="158" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A158" t="s">
         <v>13</v>
       </c>
@@ -3974,7 +3986,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="159" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A159" t="s">
         <v>13</v>
       </c>
@@ -3994,7 +4006,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="160" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A160" t="s">
         <v>13</v>
       </c>
@@ -4014,7 +4026,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="161" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A161" t="s">
         <v>13</v>
       </c>
@@ -4034,7 +4046,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="162" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A162" t="s">
         <v>13</v>
       </c>
@@ -4054,7 +4066,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="163" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A163" t="s">
         <v>13</v>
       </c>
@@ -4074,7 +4086,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="164" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A164" t="s">
         <v>13</v>
       </c>
@@ -4094,7 +4106,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="165" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A165" t="s">
         <v>13</v>
       </c>
@@ -4114,7 +4126,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="166" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A166" t="s">
         <v>13</v>
       </c>
@@ -4134,7 +4146,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="167" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A167" t="s">
         <v>13</v>
       </c>
@@ -4154,7 +4166,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="168" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A168" t="s">
         <v>13</v>
       </c>
@@ -4174,7 +4186,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="169" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A169" t="s">
         <v>13</v>
       </c>
@@ -4194,7 +4206,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="170" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A170" t="s">
         <v>13</v>
       </c>
@@ -4214,7 +4226,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="171" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A171" t="s">
         <v>13</v>
       </c>
@@ -4234,7 +4246,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="172" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A172" t="s">
         <v>13</v>
       </c>
@@ -4254,7 +4266,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="173" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A173" t="s">
         <v>13</v>
       </c>
@@ -4274,7 +4286,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="174" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A174" t="s">
         <v>13</v>
       </c>
@@ -4294,7 +4306,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="175" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A175" t="s">
         <v>13</v>
       </c>
@@ -4314,7 +4326,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="176" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A176" t="s">
         <v>13</v>
       </c>
@@ -4334,7 +4346,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="177" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A177" t="s">
         <v>13</v>
       </c>
@@ -4354,7 +4366,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="178" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A178" t="s">
         <v>13</v>
       </c>
@@ -4374,7 +4386,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="179" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A179" t="s">
         <v>13</v>
       </c>
@@ -4394,7 +4406,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="180" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A180" t="s">
         <v>13</v>
       </c>
@@ -4414,7 +4426,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="181" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A181" t="s">
         <v>13</v>
       </c>
@@ -4434,7 +4446,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="182" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A182" t="s">
         <v>13</v>
       </c>
@@ -4454,7 +4466,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="183" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A183" t="s">
         <v>13</v>
       </c>
@@ -4474,7 +4486,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="184" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A184" t="s">
         <v>13</v>
       </c>
@@ -4494,7 +4506,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="185" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A185" t="s">
         <v>13</v>
       </c>
@@ -4514,7 +4526,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="186" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A186" t="s">
         <v>13</v>
       </c>
@@ -4534,7 +4546,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="187" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A187" t="s">
         <v>13</v>
       </c>
@@ -4554,7 +4566,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="188" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A188" t="s">
         <v>13</v>
       </c>
@@ -4574,7 +4586,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="189" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A189" t="s">
         <v>13</v>
       </c>
@@ -4594,7 +4606,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="190" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A190" t="s">
         <v>13</v>
       </c>
@@ -4614,7 +4626,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="191" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A191" t="s">
         <v>13</v>
       </c>
@@ -4634,7 +4646,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="192" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A192" t="s">
         <v>13</v>
       </c>
@@ -4654,7 +4666,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="193" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A193" t="s">
         <v>13</v>
       </c>
@@ -4674,7 +4686,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="194" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A194" t="s">
         <v>14</v>
       </c>
@@ -4693,11 +4705,14 @@
       <c r="G194" t="s">
         <v>9</v>
       </c>
+      <c r="H194" t="s">
+        <v>19</v>
+      </c>
       <c r="I194" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="195" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A195" t="s">
         <v>14</v>
       </c>
@@ -4720,7 +4735,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="196" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A196" t="s">
         <v>14</v>
       </c>
@@ -4743,7 +4758,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="197" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A197" t="s">
         <v>14</v>
       </c>
@@ -4766,7 +4781,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="198" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A198" t="s">
         <v>14</v>
       </c>
@@ -4789,7 +4804,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="199" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A199" t="s">
         <v>14</v>
       </c>
@@ -4812,7 +4827,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="200" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A200" t="s">
         <v>14</v>
       </c>
@@ -4835,7 +4850,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="201" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A201" t="s">
         <v>14</v>
       </c>
@@ -4858,7 +4873,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="202" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A202" t="s">
         <v>14</v>
       </c>
@@ -4881,7 +4896,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="203" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A203" t="s">
         <v>14</v>
       </c>
@@ -4904,7 +4919,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="204" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A204" t="s">
         <v>14</v>
       </c>
@@ -4927,7 +4942,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="205" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A205" t="s">
         <v>14</v>
       </c>
@@ -4950,7 +4965,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="206" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A206" t="s">
         <v>14</v>
       </c>
@@ -4973,7 +4988,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="207" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A207" t="s">
         <v>14</v>
       </c>
@@ -4996,7 +5011,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="208" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A208" t="s">
         <v>14</v>
       </c>
@@ -5019,7 +5034,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="209" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A209" t="s">
         <v>14</v>
       </c>
@@ -5042,7 +5057,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="210" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A210" t="s">
         <v>14</v>
       </c>
@@ -5065,7 +5080,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="211" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A211" t="s">
         <v>14</v>
       </c>
@@ -5088,7 +5103,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="212" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A212" t="s">
         <v>14</v>
       </c>
@@ -5111,7 +5126,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="213" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A213" t="s">
         <v>14</v>
       </c>
@@ -5134,7 +5149,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="214" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A214" t="s">
         <v>14</v>
       </c>
@@ -5157,7 +5172,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="215" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A215" t="s">
         <v>14</v>
       </c>
@@ -5180,7 +5195,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="216" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A216" t="s">
         <v>14</v>
       </c>
@@ -5203,7 +5218,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="217" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A217" t="s">
         <v>14</v>
       </c>
@@ -5226,7 +5241,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="218" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A218" t="s">
         <v>14</v>
       </c>
@@ -5249,7 +5264,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="219" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A219" t="s">
         <v>14</v>
       </c>
@@ -5272,7 +5287,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="220" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A220" t="s">
         <v>14</v>
       </c>
@@ -5295,7 +5310,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="221" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A221" t="s">
         <v>14</v>
       </c>
@@ -5318,7 +5333,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="222" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A222" t="s">
         <v>14</v>
       </c>
@@ -5341,7 +5356,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="223" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A223" t="s">
         <v>14</v>
       </c>
@@ -5364,7 +5379,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="224" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A224" t="s">
         <v>14</v>
       </c>
@@ -5387,7 +5402,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="225" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A225" t="s">
         <v>14</v>
       </c>
@@ -5410,7 +5425,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="226" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A226" t="s">
         <v>14</v>
       </c>
@@ -5433,7 +5448,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="227" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A227" t="s">
         <v>14</v>
       </c>
@@ -5456,7 +5471,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="228" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A228" t="s">
         <v>14</v>
       </c>
@@ -5479,7 +5494,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="229" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A229" t="s">
         <v>14</v>
       </c>
@@ -5502,7 +5517,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="230" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A230" t="s">
         <v>14</v>
       </c>
@@ -5525,7 +5540,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="231" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A231" t="s">
         <v>14</v>
       </c>
@@ -5548,7 +5563,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="232" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A232" t="s">
         <v>14</v>
       </c>
@@ -5571,7 +5586,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="233" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A233" t="s">
         <v>14</v>
       </c>
@@ -5594,7 +5609,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="234" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A234" t="s">
         <v>14</v>
       </c>
@@ -5617,7 +5632,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="235" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A235" t="s">
         <v>14</v>
       </c>
@@ -5640,7 +5655,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="236" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A236" t="s">
         <v>14</v>
       </c>
@@ -5663,7 +5678,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="237" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A237" t="s">
         <v>14</v>
       </c>
@@ -5686,7 +5701,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="238" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A238" t="s">
         <v>14</v>
       </c>
@@ -5709,7 +5724,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="239" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A239" t="s">
         <v>14</v>
       </c>
@@ -5732,7 +5747,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="240" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A240" t="s">
         <v>14</v>
       </c>
@@ -5755,7 +5770,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="241" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A241" t="s">
         <v>14</v>
       </c>
@@ -5778,7 +5793,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="242" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A242" t="s">
         <v>14</v>
       </c>
@@ -5801,7 +5816,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="243" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A243" t="s">
         <v>14</v>
       </c>
@@ -5824,7 +5839,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="244" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A244" t="s">
         <v>14</v>
       </c>
@@ -5847,7 +5862,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="245" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A245" t="s">
         <v>14</v>
       </c>
@@ -5870,7 +5885,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="246" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A246" t="s">
         <v>14</v>
       </c>
@@ -5893,7 +5908,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="247" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="247" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A247" t="s">
         <v>14</v>
       </c>
@@ -5916,7 +5931,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="248" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="248" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A248" t="s">
         <v>14</v>
       </c>
@@ -5939,7 +5954,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="249" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="249" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A249" t="s">
         <v>14</v>
       </c>
@@ -5962,7 +5977,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="250" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="250" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A250" t="s">
         <v>14</v>
       </c>
@@ -5985,7 +6000,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="251" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A251" t="s">
         <v>14</v>
       </c>
@@ -6008,7 +6023,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="252" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="252" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A252" t="s">
         <v>14</v>
       </c>
@@ -6031,7 +6046,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="253" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="253" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A253" t="s">
         <v>14</v>
       </c>
@@ -6054,7 +6069,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="254" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="254" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A254" t="s">
         <v>14</v>
       </c>
@@ -6077,7 +6092,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="255" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="255" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A255" t="s">
         <v>14</v>
       </c>
@@ -6100,7 +6115,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="256" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="256" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A256" t="s">
         <v>14</v>
       </c>
@@ -6123,7 +6138,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="257" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="257" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A257" t="s">
         <v>14</v>
       </c>
@@ -6146,7 +6161,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="258" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="258" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A258" t="s">
         <v>16</v>
       </c>
@@ -6165,11 +6180,14 @@
       <c r="G258" t="s">
         <v>9</v>
       </c>
+      <c r="H258" t="s">
+        <v>18</v>
+      </c>
       <c r="I258" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="259" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="259" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A259" t="s">
         <v>16</v>
       </c>
@@ -6192,7 +6210,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="260" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="260" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A260" t="s">
         <v>16</v>
       </c>
@@ -6215,7 +6233,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="261" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="261" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A261" t="s">
         <v>16</v>
       </c>
@@ -6238,7 +6256,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="262" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="262" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A262" t="s">
         <v>16</v>
       </c>
@@ -6261,7 +6279,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="263" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="263" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A263" t="s">
         <v>16</v>
       </c>
@@ -6284,7 +6302,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="264" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="264" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A264" t="s">
         <v>16</v>
       </c>
@@ -6307,7 +6325,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="265" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="265" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A265" t="s">
         <v>16</v>
       </c>
@@ -6330,7 +6348,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="266" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="266" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A266" t="s">
         <v>16</v>
       </c>
@@ -6353,7 +6371,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="267" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="267" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A267" t="s">
         <v>16</v>
       </c>
@@ -6376,7 +6394,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="268" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="268" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A268" t="s">
         <v>16</v>
       </c>
@@ -6399,7 +6417,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="269" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="269" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A269" t="s">
         <v>16</v>
       </c>
@@ -6422,7 +6440,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="270" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="270" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A270" t="s">
         <v>16</v>
       </c>
@@ -6445,7 +6463,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="271" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="271" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A271" t="s">
         <v>16</v>
       </c>
@@ -6468,7 +6486,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="272" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="272" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A272" t="s">
         <v>16</v>
       </c>
@@ -6491,7 +6509,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="273" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="273" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A273" t="s">
         <v>16</v>
       </c>
@@ -6514,7 +6532,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="274" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="274" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A274" t="s">
         <v>16</v>
       </c>
@@ -6537,7 +6555,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="275" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="275" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A275" t="s">
         <v>16</v>
       </c>
@@ -6560,7 +6578,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="276" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="276" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A276" t="s">
         <v>16</v>
       </c>
@@ -6583,7 +6601,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="277" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="277" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A277" t="s">
         <v>16</v>
       </c>
@@ -6606,7 +6624,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="278" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="278" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A278" t="s">
         <v>16</v>
       </c>
@@ -6629,7 +6647,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="279" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="279" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A279" t="s">
         <v>16</v>
       </c>
@@ -6652,7 +6670,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="280" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="280" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A280" t="s">
         <v>16</v>
       </c>
@@ -6675,7 +6693,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="281" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="281" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A281" t="s">
         <v>16</v>
       </c>
@@ -6698,7 +6716,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="282" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="282" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A282" t="s">
         <v>16</v>
       </c>
@@ -6721,7 +6739,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="283" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="283" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A283" t="s">
         <v>16</v>
       </c>
@@ -6744,7 +6762,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="284" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="284" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A284" t="s">
         <v>16</v>
       </c>
@@ -6767,7 +6785,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="285" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="285" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A285" t="s">
         <v>16</v>
       </c>
@@ -6790,7 +6808,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="286" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="286" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A286" t="s">
         <v>16</v>
       </c>
@@ -6813,7 +6831,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="287" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="287" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A287" t="s">
         <v>16</v>
       </c>
@@ -6836,7 +6854,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="288" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="288" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A288" t="s">
         <v>16</v>
       </c>
@@ -6859,7 +6877,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="289" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="289" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A289" t="s">
         <v>16</v>
       </c>
@@ -6882,7 +6900,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="290" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="290" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A290" t="s">
         <v>16</v>
       </c>
@@ -6905,7 +6923,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="291" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="291" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A291" t="s">
         <v>16</v>
       </c>
@@ -6928,7 +6946,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="292" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="292" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A292" t="s">
         <v>16</v>
       </c>
@@ -6951,7 +6969,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="293" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="293" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A293" t="s">
         <v>16</v>
       </c>
@@ -6974,7 +6992,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="294" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="294" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A294" t="s">
         <v>16</v>
       </c>
@@ -6997,7 +7015,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="295" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="295" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A295" t="s">
         <v>16</v>
       </c>
@@ -7020,7 +7038,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="296" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="296" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A296" t="s">
         <v>16</v>
       </c>
@@ -7043,7 +7061,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="297" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="297" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A297" t="s">
         <v>16</v>
       </c>
@@ -7066,7 +7084,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="298" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="298" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A298" t="s">
         <v>16</v>
       </c>
@@ -7089,7 +7107,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="299" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="299" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A299" t="s">
         <v>16</v>
       </c>
@@ -7112,7 +7130,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="300" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="300" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A300" t="s">
         <v>16</v>
       </c>
@@ -7135,7 +7153,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="301" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="301" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A301" t="s">
         <v>16</v>
       </c>
@@ -7158,7 +7176,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="302" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="302" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A302" t="s">
         <v>16</v>
       </c>
@@ -7181,7 +7199,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="303" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="303" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A303" t="s">
         <v>16</v>
       </c>
@@ -7204,7 +7222,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="304" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="304" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A304" t="s">
         <v>16</v>
       </c>
@@ -7227,7 +7245,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="305" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="305" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A305" t="s">
         <v>16</v>
       </c>
@@ -7250,7 +7268,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="306" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="306" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A306" t="s">
         <v>16</v>
       </c>
@@ -7273,7 +7291,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="307" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="307" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A307" t="s">
         <v>16</v>
       </c>
@@ -7296,7 +7314,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="308" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="308" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A308" t="s">
         <v>16</v>
       </c>
@@ -7319,7 +7337,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="309" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="309" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A309" t="s">
         <v>16</v>
       </c>
@@ -7342,7 +7360,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="310" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="310" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A310" t="s">
         <v>16</v>
       </c>
@@ -7365,7 +7383,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="311" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="311" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A311" t="s">
         <v>16</v>
       </c>
@@ -7388,7 +7406,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="312" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="312" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A312" t="s">
         <v>16</v>
       </c>
@@ -7411,7 +7429,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="313" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="313" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A313" t="s">
         <v>16</v>
       </c>
@@ -7434,7 +7452,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="314" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="314" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A314" t="s">
         <v>16</v>
       </c>
@@ -7457,7 +7475,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="315" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="315" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A315" t="s">
         <v>16</v>
       </c>
@@ -7480,7 +7498,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="316" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="316" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A316" t="s">
         <v>16</v>
       </c>
@@ -7503,7 +7521,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="317" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="317" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A317" t="s">
         <v>16</v>
       </c>
@@ -7526,7 +7544,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="318" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="318" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A318" t="s">
         <v>16</v>
       </c>
@@ -7549,7 +7567,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="319" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="319" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A319" t="s">
         <v>16</v>
       </c>
@@ -7572,7 +7590,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="320" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="320" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A320" t="s">
         <v>16</v>
       </c>
@@ -7595,7 +7613,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="321" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="321" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A321" t="s">
         <v>16</v>
       </c>
@@ -7624,7 +7642,7 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:I193 A194:A321 I194:I321" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:I129 A194:A321 I194:I321 A131:I193 A130:G130 I130" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
One excel for mens and womens results
</commit_message>
<xml_diff>
--- a/pages/video_analysis/IP_Master_Men.xlsx
+++ b/pages/video_analysis/IP_Master_Men.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sportnzgroup-my.sharepoint.com/personal/anja_kuys_hpsnz_org_nz/Documents/Desktop/Scripts/CNZPD/pages/video_analysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="11_F1FC6792D89E629903ED24B2C9460C765188C8B3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D2D1CB14-47C1-4953-96E7-B64BD2730C23}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="11_F1FC6792D89E629903ED24B2C9460C765188C8B3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2FD742A7-85B4-4B4C-A004-06A21C31CBA8}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="1620" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="778" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="781" uniqueCount="20">
   <si>
     <t>Title</t>
   </si>
@@ -71,6 +71,15 @@
   </si>
   <si>
     <t>26-07-31 Glasgow CWG Morton Q</t>
+  </si>
+  <si>
+    <t>https://youtu.be/qCTIxXtG0Lg</t>
+  </si>
+  <si>
+    <t>https://youtu.be/yjVZcfO11qw</t>
+  </si>
+  <si>
+    <t>https://youtu.be/z7zcj4I4qic</t>
   </si>
 </sst>
 </file>
@@ -413,12 +422,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I321"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="32.58203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -444,7 +453,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -470,7 +479,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -493,7 +502,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -516,7 +525,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -539,7 +548,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -562,7 +571,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -585,7 +594,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -608,7 +617,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -631,7 +640,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -654,7 +663,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>8</v>
       </c>
@@ -677,7 +686,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>8</v>
       </c>
@@ -700,7 +709,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>8</v>
       </c>
@@ -723,7 +732,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>8</v>
       </c>
@@ -746,7 +755,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>8</v>
       </c>
@@ -769,7 +778,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>8</v>
       </c>
@@ -792,7 +801,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>8</v>
       </c>
@@ -815,7 +824,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>8</v>
       </c>
@@ -838,7 +847,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>8</v>
       </c>
@@ -861,7 +870,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>8</v>
       </c>
@@ -884,7 +893,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>8</v>
       </c>
@@ -907,7 +916,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>8</v>
       </c>
@@ -930,7 +939,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="23" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>8</v>
       </c>
@@ -953,7 +962,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>8</v>
       </c>
@@ -976,7 +985,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="25" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>8</v>
       </c>
@@ -999,7 +1008,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>8</v>
       </c>
@@ -1022,7 +1031,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="27" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>8</v>
       </c>
@@ -1045,7 +1054,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="28" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>8</v>
       </c>
@@ -1068,7 +1077,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="29" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>8</v>
       </c>
@@ -1091,7 +1100,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="30" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>8</v>
       </c>
@@ -1114,7 +1123,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="31" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>8</v>
       </c>
@@ -1137,7 +1146,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="32" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>8</v>
       </c>
@@ -1160,7 +1169,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="33" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>8</v>
       </c>
@@ -1183,7 +1192,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="34" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>8</v>
       </c>
@@ -1206,7 +1215,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="35" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>8</v>
       </c>
@@ -1229,7 +1238,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="36" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>8</v>
       </c>
@@ -1252,7 +1261,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="37" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>8</v>
       </c>
@@ -1275,7 +1284,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="38" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>8</v>
       </c>
@@ -1298,7 +1307,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="39" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>8</v>
       </c>
@@ -1321,7 +1330,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="40" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>8</v>
       </c>
@@ -1344,7 +1353,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="41" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>8</v>
       </c>
@@ -1367,7 +1376,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="42" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>8</v>
       </c>
@@ -1390,7 +1399,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="43" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>8</v>
       </c>
@@ -1413,7 +1422,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="44" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>8</v>
       </c>
@@ -1436,7 +1445,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="45" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>8</v>
       </c>
@@ -1459,7 +1468,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="46" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>8</v>
       </c>
@@ -1482,7 +1491,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="47" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>8</v>
       </c>
@@ -1505,7 +1514,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="48" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>8</v>
       </c>
@@ -1528,7 +1537,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="49" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>8</v>
       </c>
@@ -1551,7 +1560,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="50" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>8</v>
       </c>
@@ -1574,7 +1583,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="51" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>8</v>
       </c>
@@ -1597,7 +1606,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="52" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>8</v>
       </c>
@@ -1620,7 +1629,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="53" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>8</v>
       </c>
@@ -1643,7 +1652,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="54" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>8</v>
       </c>
@@ -1666,7 +1675,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="55" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>8</v>
       </c>
@@ -1689,7 +1698,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="56" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>8</v>
       </c>
@@ -1712,7 +1721,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="57" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>8</v>
       </c>
@@ -1735,7 +1744,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="58" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>8</v>
       </c>
@@ -1758,7 +1767,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="59" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>8</v>
       </c>
@@ -1781,7 +1790,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="60" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>8</v>
       </c>
@@ -1804,7 +1813,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="61" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>8</v>
       </c>
@@ -1827,7 +1836,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="62" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>8</v>
       </c>
@@ -1850,7 +1859,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="63" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>8</v>
       </c>
@@ -1873,7 +1882,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="64" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>8</v>
       </c>
@@ -1896,7 +1905,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="65" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>8</v>
       </c>
@@ -1919,7 +1928,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="66" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>11</v>
       </c>
@@ -1945,7 +1954,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="67" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>11</v>
       </c>
@@ -1968,7 +1977,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="68" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>11</v>
       </c>
@@ -1991,7 +2000,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="69" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>11</v>
       </c>
@@ -2014,7 +2023,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="70" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>11</v>
       </c>
@@ -2037,7 +2046,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="71" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>11</v>
       </c>
@@ -2060,7 +2069,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="72" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>11</v>
       </c>
@@ -2083,7 +2092,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="73" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>11</v>
       </c>
@@ -2106,7 +2115,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="74" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>11</v>
       </c>
@@ -2129,7 +2138,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="75" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>11</v>
       </c>
@@ -2152,7 +2161,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="76" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>11</v>
       </c>
@@ -2175,7 +2184,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="77" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>11</v>
       </c>
@@ -2198,7 +2207,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="78" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>11</v>
       </c>
@@ -2221,7 +2230,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="79" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>11</v>
       </c>
@@ -2244,7 +2253,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="80" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>11</v>
       </c>
@@ -2267,7 +2276,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="81" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>11</v>
       </c>
@@ -2290,7 +2299,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="82" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>11</v>
       </c>
@@ -2313,7 +2322,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="83" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>11</v>
       </c>
@@ -2336,7 +2345,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="84" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>11</v>
       </c>
@@ -2359,7 +2368,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="85" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>11</v>
       </c>
@@ -2382,7 +2391,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="86" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>11</v>
       </c>
@@ -2405,7 +2414,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="87" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>11</v>
       </c>
@@ -2428,7 +2437,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="88" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>11</v>
       </c>
@@ -2451,7 +2460,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="89" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>11</v>
       </c>
@@ -2474,7 +2483,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="90" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>11</v>
       </c>
@@ -2497,7 +2506,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="91" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>11</v>
       </c>
@@ -2520,7 +2529,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="92" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>11</v>
       </c>
@@ -2543,7 +2552,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="93" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>11</v>
       </c>
@@ -2566,7 +2575,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="94" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>11</v>
       </c>
@@ -2589,7 +2598,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="95" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>11</v>
       </c>
@@ -2612,7 +2621,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="96" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>11</v>
       </c>
@@ -2635,7 +2644,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="97" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>11</v>
       </c>
@@ -2658,7 +2667,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="98" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
         <v>11</v>
       </c>
@@ -2681,7 +2690,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="99" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
         <v>11</v>
       </c>
@@ -2704,7 +2713,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="100" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
         <v>11</v>
       </c>
@@ -2727,7 +2736,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="101" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
         <v>11</v>
       </c>
@@ -2750,7 +2759,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="102" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
         <v>11</v>
       </c>
@@ -2773,7 +2782,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="103" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
         <v>11</v>
       </c>
@@ -2796,7 +2805,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="104" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
         <v>11</v>
       </c>
@@ -2819,7 +2828,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="105" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
         <v>11</v>
       </c>
@@ -2842,7 +2851,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="106" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
         <v>11</v>
       </c>
@@ -2865,7 +2874,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="107" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
         <v>11</v>
       </c>
@@ -2888,7 +2897,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="108" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
         <v>11</v>
       </c>
@@ -2911,7 +2920,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="109" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
         <v>11</v>
       </c>
@@ -2934,7 +2943,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="110" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
         <v>11</v>
       </c>
@@ -2957,7 +2966,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="111" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
         <v>11</v>
       </c>
@@ -2980,7 +2989,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="112" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
         <v>11</v>
       </c>
@@ -3003,7 +3012,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="113" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
         <v>11</v>
       </c>
@@ -3026,7 +3035,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="114" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
         <v>11</v>
       </c>
@@ -3049,7 +3058,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="115" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
         <v>11</v>
       </c>
@@ -3072,7 +3081,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="116" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
         <v>11</v>
       </c>
@@ -3095,7 +3104,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="117" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
         <v>11</v>
       </c>
@@ -3118,7 +3127,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="118" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
         <v>11</v>
       </c>
@@ -3141,7 +3150,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="119" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
         <v>11</v>
       </c>
@@ -3164,7 +3173,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="120" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
         <v>11</v>
       </c>
@@ -3187,7 +3196,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="121" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
         <v>11</v>
       </c>
@@ -3210,7 +3219,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="122" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
         <v>11</v>
       </c>
@@ -3233,7 +3242,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="123" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
         <v>11</v>
       </c>
@@ -3256,7 +3265,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="124" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A124" t="s">
         <v>11</v>
       </c>
@@ -3279,7 +3288,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="125" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
         <v>11</v>
       </c>
@@ -3302,7 +3311,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="126" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A126" t="s">
         <v>11</v>
       </c>
@@ -3325,7 +3334,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="127" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A127" t="s">
         <v>11</v>
       </c>
@@ -3348,7 +3357,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="128" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A128" t="s">
         <v>11</v>
       </c>
@@ -3371,7 +3380,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="129" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A129" t="s">
         <v>11</v>
       </c>
@@ -3394,7 +3403,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="130" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A130" t="s">
         <v>13</v>
       </c>
@@ -3413,8 +3422,11 @@
       <c r="G130" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="131" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="H130" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="131" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A131" t="s">
         <v>13</v>
       </c>
@@ -3434,7 +3446,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="132" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A132" t="s">
         <v>13</v>
       </c>
@@ -3454,7 +3466,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="133" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A133" t="s">
         <v>13</v>
       </c>
@@ -3474,7 +3486,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="134" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A134" t="s">
         <v>13</v>
       </c>
@@ -3494,7 +3506,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="135" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A135" t="s">
         <v>13</v>
       </c>
@@ -3514,7 +3526,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="136" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A136" t="s">
         <v>13</v>
       </c>
@@ -3534,7 +3546,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="137" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A137" t="s">
         <v>13</v>
       </c>
@@ -3554,7 +3566,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="138" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A138" t="s">
         <v>13</v>
       </c>
@@ -3574,7 +3586,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="139" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A139" t="s">
         <v>13</v>
       </c>
@@ -3594,7 +3606,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="140" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A140" t="s">
         <v>13</v>
       </c>
@@ -3614,7 +3626,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="141" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A141" t="s">
         <v>13</v>
       </c>
@@ -3634,7 +3646,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="142" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A142" t="s">
         <v>13</v>
       </c>
@@ -3654,7 +3666,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="143" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A143" t="s">
         <v>13</v>
       </c>
@@ -3674,7 +3686,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="144" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A144" t="s">
         <v>13</v>
       </c>
@@ -3694,7 +3706,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="145" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A145" t="s">
         <v>13</v>
       </c>
@@ -3714,7 +3726,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="146" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A146" t="s">
         <v>13</v>
       </c>
@@ -3734,7 +3746,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="147" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A147" t="s">
         <v>13</v>
       </c>
@@ -3754,7 +3766,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="148" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A148" t="s">
         <v>13</v>
       </c>
@@ -3774,7 +3786,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="149" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A149" t="s">
         <v>13</v>
       </c>
@@ -3794,7 +3806,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="150" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A150" t="s">
         <v>13</v>
       </c>
@@ -3814,7 +3826,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="151" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A151" t="s">
         <v>13</v>
       </c>
@@ -3834,7 +3846,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="152" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A152" t="s">
         <v>13</v>
       </c>
@@ -3854,7 +3866,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="153" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A153" t="s">
         <v>13</v>
       </c>
@@ -3874,7 +3886,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="154" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A154" t="s">
         <v>13</v>
       </c>
@@ -3894,7 +3906,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="155" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A155" t="s">
         <v>13</v>
       </c>
@@ -3914,7 +3926,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="156" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A156" t="s">
         <v>13</v>
       </c>
@@ -3934,7 +3946,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="157" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A157" t="s">
         <v>13</v>
       </c>
@@ -3954,7 +3966,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="158" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A158" t="s">
         <v>13</v>
       </c>
@@ -3974,7 +3986,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="159" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A159" t="s">
         <v>13</v>
       </c>
@@ -3994,7 +4006,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="160" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A160" t="s">
         <v>13</v>
       </c>
@@ -4014,7 +4026,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="161" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A161" t="s">
         <v>13</v>
       </c>
@@ -4034,7 +4046,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="162" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A162" t="s">
         <v>13</v>
       </c>
@@ -4054,7 +4066,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="163" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A163" t="s">
         <v>13</v>
       </c>
@@ -4074,7 +4086,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="164" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A164" t="s">
         <v>13</v>
       </c>
@@ -4094,7 +4106,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="165" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A165" t="s">
         <v>13</v>
       </c>
@@ -4114,7 +4126,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="166" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A166" t="s">
         <v>13</v>
       </c>
@@ -4134,7 +4146,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="167" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A167" t="s">
         <v>13</v>
       </c>
@@ -4154,7 +4166,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="168" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A168" t="s">
         <v>13</v>
       </c>
@@ -4174,7 +4186,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="169" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A169" t="s">
         <v>13</v>
       </c>
@@ -4194,7 +4206,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="170" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A170" t="s">
         <v>13</v>
       </c>
@@ -4214,7 +4226,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="171" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A171" t="s">
         <v>13</v>
       </c>
@@ -4234,7 +4246,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="172" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A172" t="s">
         <v>13</v>
       </c>
@@ -4254,7 +4266,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="173" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A173" t="s">
         <v>13</v>
       </c>
@@ -4274,7 +4286,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="174" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A174" t="s">
         <v>13</v>
       </c>
@@ -4294,7 +4306,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="175" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A175" t="s">
         <v>13</v>
       </c>
@@ -4314,7 +4326,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="176" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A176" t="s">
         <v>13</v>
       </c>
@@ -4334,7 +4346,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="177" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A177" t="s">
         <v>13</v>
       </c>
@@ -4354,7 +4366,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="178" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A178" t="s">
         <v>13</v>
       </c>
@@ -4374,7 +4386,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="179" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A179" t="s">
         <v>13</v>
       </c>
@@ -4394,7 +4406,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="180" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A180" t="s">
         <v>13</v>
       </c>
@@ -4414,7 +4426,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="181" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A181" t="s">
         <v>13</v>
       </c>
@@ -4434,7 +4446,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="182" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A182" t="s">
         <v>13</v>
       </c>
@@ -4454,7 +4466,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="183" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A183" t="s">
         <v>13</v>
       </c>
@@ -4474,7 +4486,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="184" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A184" t="s">
         <v>13</v>
       </c>
@@ -4494,7 +4506,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="185" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A185" t="s">
         <v>13</v>
       </c>
@@ -4514,7 +4526,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="186" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A186" t="s">
         <v>13</v>
       </c>
@@ -4534,7 +4546,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="187" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A187" t="s">
         <v>13</v>
       </c>
@@ -4554,7 +4566,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="188" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A188" t="s">
         <v>13</v>
       </c>
@@ -4574,7 +4586,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="189" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A189" t="s">
         <v>13</v>
       </c>
@@ -4594,7 +4606,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="190" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A190" t="s">
         <v>13</v>
       </c>
@@ -4614,7 +4626,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="191" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A191" t="s">
         <v>13</v>
       </c>
@@ -4634,7 +4646,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="192" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A192" t="s">
         <v>13</v>
       </c>
@@ -4654,7 +4666,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="193" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A193" t="s">
         <v>13</v>
       </c>
@@ -4674,7 +4686,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="194" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A194" t="s">
         <v>14</v>
       </c>
@@ -4693,11 +4705,14 @@
       <c r="G194" t="s">
         <v>9</v>
       </c>
+      <c r="H194" t="s">
+        <v>19</v>
+      </c>
       <c r="I194" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="195" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A195" t="s">
         <v>14</v>
       </c>
@@ -4720,7 +4735,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="196" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A196" t="s">
         <v>14</v>
       </c>
@@ -4743,7 +4758,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="197" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A197" t="s">
         <v>14</v>
       </c>
@@ -4766,7 +4781,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="198" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A198" t="s">
         <v>14</v>
       </c>
@@ -4789,7 +4804,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="199" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A199" t="s">
         <v>14</v>
       </c>
@@ -4812,7 +4827,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="200" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A200" t="s">
         <v>14</v>
       </c>
@@ -4835,7 +4850,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="201" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A201" t="s">
         <v>14</v>
       </c>
@@ -4858,7 +4873,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="202" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A202" t="s">
         <v>14</v>
       </c>
@@ -4881,7 +4896,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="203" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A203" t="s">
         <v>14</v>
       </c>
@@ -4904,7 +4919,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="204" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A204" t="s">
         <v>14</v>
       </c>
@@ -4927,7 +4942,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="205" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A205" t="s">
         <v>14</v>
       </c>
@@ -4950,7 +4965,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="206" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A206" t="s">
         <v>14</v>
       </c>
@@ -4973,7 +4988,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="207" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A207" t="s">
         <v>14</v>
       </c>
@@ -4996,7 +5011,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="208" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A208" t="s">
         <v>14</v>
       </c>
@@ -5019,7 +5034,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="209" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A209" t="s">
         <v>14</v>
       </c>
@@ -5042,7 +5057,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="210" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A210" t="s">
         <v>14</v>
       </c>
@@ -5065,7 +5080,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="211" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A211" t="s">
         <v>14</v>
       </c>
@@ -5088,7 +5103,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="212" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A212" t="s">
         <v>14</v>
       </c>
@@ -5111,7 +5126,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="213" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A213" t="s">
         <v>14</v>
       </c>
@@ -5134,7 +5149,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="214" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A214" t="s">
         <v>14</v>
       </c>
@@ -5157,7 +5172,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="215" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A215" t="s">
         <v>14</v>
       </c>
@@ -5180,7 +5195,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="216" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A216" t="s">
         <v>14</v>
       </c>
@@ -5203,7 +5218,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="217" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A217" t="s">
         <v>14</v>
       </c>
@@ -5226,7 +5241,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="218" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A218" t="s">
         <v>14</v>
       </c>
@@ -5249,7 +5264,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="219" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A219" t="s">
         <v>14</v>
       </c>
@@ -5272,7 +5287,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="220" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A220" t="s">
         <v>14</v>
       </c>
@@ -5295,7 +5310,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="221" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A221" t="s">
         <v>14</v>
       </c>
@@ -5318,7 +5333,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="222" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A222" t="s">
         <v>14</v>
       </c>
@@ -5341,7 +5356,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="223" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A223" t="s">
         <v>14</v>
       </c>
@@ -5364,7 +5379,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="224" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A224" t="s">
         <v>14</v>
       </c>
@@ -5387,7 +5402,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="225" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A225" t="s">
         <v>14</v>
       </c>
@@ -5410,7 +5425,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="226" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A226" t="s">
         <v>14</v>
       </c>
@@ -5433,7 +5448,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="227" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A227" t="s">
         <v>14</v>
       </c>
@@ -5456,7 +5471,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="228" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A228" t="s">
         <v>14</v>
       </c>
@@ -5479,7 +5494,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="229" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A229" t="s">
         <v>14</v>
       </c>
@@ -5502,7 +5517,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="230" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A230" t="s">
         <v>14</v>
       </c>
@@ -5525,7 +5540,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="231" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A231" t="s">
         <v>14</v>
       </c>
@@ -5548,7 +5563,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="232" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A232" t="s">
         <v>14</v>
       </c>
@@ -5571,7 +5586,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="233" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A233" t="s">
         <v>14</v>
       </c>
@@ -5594,7 +5609,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="234" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A234" t="s">
         <v>14</v>
       </c>
@@ -5617,7 +5632,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="235" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A235" t="s">
         <v>14</v>
       </c>
@@ -5640,7 +5655,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="236" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A236" t="s">
         <v>14</v>
       </c>
@@ -5663,7 +5678,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="237" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A237" t="s">
         <v>14</v>
       </c>
@@ -5686,7 +5701,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="238" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A238" t="s">
         <v>14</v>
       </c>
@@ -5709,7 +5724,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="239" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A239" t="s">
         <v>14</v>
       </c>
@@ -5732,7 +5747,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="240" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A240" t="s">
         <v>14</v>
       </c>
@@ -5755,7 +5770,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="241" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A241" t="s">
         <v>14</v>
       </c>
@@ -5778,7 +5793,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="242" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A242" t="s">
         <v>14</v>
       </c>
@@ -5801,7 +5816,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="243" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A243" t="s">
         <v>14</v>
       </c>
@@ -5824,7 +5839,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="244" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A244" t="s">
         <v>14</v>
       </c>
@@ -5847,7 +5862,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="245" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A245" t="s">
         <v>14</v>
       </c>
@@ -5870,7 +5885,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="246" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A246" t="s">
         <v>14</v>
       </c>
@@ -5893,7 +5908,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="247" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="247" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A247" t="s">
         <v>14</v>
       </c>
@@ -5916,7 +5931,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="248" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="248" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A248" t="s">
         <v>14</v>
       </c>
@@ -5939,7 +5954,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="249" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="249" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A249" t="s">
         <v>14</v>
       </c>
@@ -5962,7 +5977,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="250" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="250" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A250" t="s">
         <v>14</v>
       </c>
@@ -5985,7 +6000,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="251" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A251" t="s">
         <v>14</v>
       </c>
@@ -6008,7 +6023,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="252" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="252" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A252" t="s">
         <v>14</v>
       </c>
@@ -6031,7 +6046,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="253" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="253" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A253" t="s">
         <v>14</v>
       </c>
@@ -6054,7 +6069,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="254" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="254" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A254" t="s">
         <v>14</v>
       </c>
@@ -6077,7 +6092,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="255" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="255" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A255" t="s">
         <v>14</v>
       </c>
@@ -6100,7 +6115,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="256" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="256" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A256" t="s">
         <v>14</v>
       </c>
@@ -6123,7 +6138,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="257" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="257" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A257" t="s">
         <v>14</v>
       </c>
@@ -6146,7 +6161,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="258" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="258" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A258" t="s">
         <v>16</v>
       </c>
@@ -6165,11 +6180,14 @@
       <c r="G258" t="s">
         <v>9</v>
       </c>
+      <c r="H258" t="s">
+        <v>18</v>
+      </c>
       <c r="I258" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="259" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="259" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A259" t="s">
         <v>16</v>
       </c>
@@ -6192,7 +6210,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="260" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="260" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A260" t="s">
         <v>16</v>
       </c>
@@ -6215,7 +6233,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="261" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="261" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A261" t="s">
         <v>16</v>
       </c>
@@ -6238,7 +6256,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="262" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="262" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A262" t="s">
         <v>16</v>
       </c>
@@ -6261,7 +6279,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="263" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="263" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A263" t="s">
         <v>16</v>
       </c>
@@ -6284,7 +6302,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="264" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="264" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A264" t="s">
         <v>16</v>
       </c>
@@ -6307,7 +6325,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="265" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="265" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A265" t="s">
         <v>16</v>
       </c>
@@ -6330,7 +6348,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="266" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="266" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A266" t="s">
         <v>16</v>
       </c>
@@ -6353,7 +6371,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="267" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="267" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A267" t="s">
         <v>16</v>
       </c>
@@ -6376,7 +6394,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="268" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="268" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A268" t="s">
         <v>16</v>
       </c>
@@ -6399,7 +6417,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="269" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="269" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A269" t="s">
         <v>16</v>
       </c>
@@ -6422,7 +6440,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="270" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="270" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A270" t="s">
         <v>16</v>
       </c>
@@ -6445,7 +6463,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="271" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="271" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A271" t="s">
         <v>16</v>
       </c>
@@ -6468,7 +6486,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="272" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="272" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A272" t="s">
         <v>16</v>
       </c>
@@ -6491,7 +6509,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="273" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="273" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A273" t="s">
         <v>16</v>
       </c>
@@ -6514,7 +6532,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="274" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="274" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A274" t="s">
         <v>16</v>
       </c>
@@ -6537,7 +6555,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="275" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="275" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A275" t="s">
         <v>16</v>
       </c>
@@ -6560,7 +6578,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="276" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="276" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A276" t="s">
         <v>16</v>
       </c>
@@ -6583,7 +6601,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="277" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="277" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A277" t="s">
         <v>16</v>
       </c>
@@ -6606,7 +6624,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="278" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="278" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A278" t="s">
         <v>16</v>
       </c>
@@ -6629,7 +6647,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="279" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="279" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A279" t="s">
         <v>16</v>
       </c>
@@ -6652,7 +6670,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="280" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="280" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A280" t="s">
         <v>16</v>
       </c>
@@ -6675,7 +6693,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="281" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="281" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A281" t="s">
         <v>16</v>
       </c>
@@ -6698,7 +6716,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="282" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="282" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A282" t="s">
         <v>16</v>
       </c>
@@ -6721,7 +6739,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="283" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="283" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A283" t="s">
         <v>16</v>
       </c>
@@ -6744,7 +6762,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="284" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="284" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A284" t="s">
         <v>16</v>
       </c>
@@ -6767,7 +6785,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="285" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="285" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A285" t="s">
         <v>16</v>
       </c>
@@ -6790,7 +6808,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="286" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="286" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A286" t="s">
         <v>16</v>
       </c>
@@ -6813,7 +6831,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="287" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="287" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A287" t="s">
         <v>16</v>
       </c>
@@ -6836,7 +6854,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="288" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="288" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A288" t="s">
         <v>16</v>
       </c>
@@ -6859,7 +6877,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="289" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="289" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A289" t="s">
         <v>16</v>
       </c>
@@ -6882,7 +6900,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="290" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="290" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A290" t="s">
         <v>16</v>
       </c>
@@ -6905,7 +6923,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="291" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="291" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A291" t="s">
         <v>16</v>
       </c>
@@ -6928,7 +6946,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="292" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="292" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A292" t="s">
         <v>16</v>
       </c>
@@ -6951,7 +6969,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="293" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="293" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A293" t="s">
         <v>16</v>
       </c>
@@ -6974,7 +6992,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="294" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="294" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A294" t="s">
         <v>16</v>
       </c>
@@ -6997,7 +7015,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="295" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="295" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A295" t="s">
         <v>16</v>
       </c>
@@ -7020,7 +7038,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="296" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="296" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A296" t="s">
         <v>16</v>
       </c>
@@ -7043,7 +7061,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="297" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="297" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A297" t="s">
         <v>16</v>
       </c>
@@ -7066,7 +7084,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="298" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="298" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A298" t="s">
         <v>16</v>
       </c>
@@ -7089,7 +7107,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="299" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="299" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A299" t="s">
         <v>16</v>
       </c>
@@ -7112,7 +7130,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="300" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="300" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A300" t="s">
         <v>16</v>
       </c>
@@ -7135,7 +7153,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="301" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="301" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A301" t="s">
         <v>16</v>
       </c>
@@ -7158,7 +7176,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="302" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="302" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A302" t="s">
         <v>16</v>
       </c>
@@ -7181,7 +7199,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="303" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="303" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A303" t="s">
         <v>16</v>
       </c>
@@ -7204,7 +7222,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="304" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="304" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A304" t="s">
         <v>16</v>
       </c>
@@ -7227,7 +7245,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="305" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="305" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A305" t="s">
         <v>16</v>
       </c>
@@ -7250,7 +7268,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="306" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="306" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A306" t="s">
         <v>16</v>
       </c>
@@ -7273,7 +7291,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="307" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="307" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A307" t="s">
         <v>16</v>
       </c>
@@ -7296,7 +7314,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="308" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="308" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A308" t="s">
         <v>16</v>
       </c>
@@ -7319,7 +7337,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="309" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="309" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A309" t="s">
         <v>16</v>
       </c>
@@ -7342,7 +7360,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="310" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="310" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A310" t="s">
         <v>16</v>
       </c>
@@ -7365,7 +7383,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="311" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="311" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A311" t="s">
         <v>16</v>
       </c>
@@ -7388,7 +7406,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="312" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="312" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A312" t="s">
         <v>16</v>
       </c>
@@ -7411,7 +7429,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="313" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="313" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A313" t="s">
         <v>16</v>
       </c>
@@ -7434,7 +7452,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="314" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="314" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A314" t="s">
         <v>16</v>
       </c>
@@ -7457,7 +7475,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="315" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="315" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A315" t="s">
         <v>16</v>
       </c>
@@ -7480,7 +7498,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="316" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="316" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A316" t="s">
         <v>16</v>
       </c>
@@ -7503,7 +7521,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="317" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="317" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A317" t="s">
         <v>16</v>
       </c>
@@ -7526,7 +7544,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="318" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="318" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A318" t="s">
         <v>16</v>
       </c>
@@ -7549,7 +7567,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="319" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="319" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A319" t="s">
         <v>16</v>
       </c>
@@ -7572,7 +7590,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="320" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="320" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A320" t="s">
         <v>16</v>
       </c>
@@ -7595,7 +7613,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="321" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="321" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A321" t="s">
         <v>16</v>
       </c>
@@ -7624,7 +7642,7 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:I193 A194:A321 I194:I321" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:I129 A194:A321 I194:I321 A131:I193 A130:G130 I130" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>